<commit_message>
test #3 workflow horarios
</commit_message>
<xml_diff>
--- a/tren-urquiza-horarios.xlsx
+++ b/tren-urquiza-horarios.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="329">
   <si>
     <t>Tren Urquiza — Lunes a Viernes → Lacroze</t>
   </si>
@@ -1238,6 +1238,9 @@
     <xf borderId="4" fillId="8" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="4" fillId="8" fontId="11" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="4" fillId="8" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -1249,9 +1252,6 @@
     </xf>
     <xf borderId="2" fillId="0" fontId="13" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="13" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="8" fontId="11" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -29183,290 +29183,290 @@
       <c r="A5" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="B5" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="C5" s="20" t="s">
+      <c r="B5" s="20">
+        <v>0.08333333333333333</v>
+      </c>
+      <c r="C5" s="21" t="s">
         <v>210</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="21" t="s">
         <v>212</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="21" t="s">
         <v>213</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="21" t="s">
         <v>214</v>
       </c>
-      <c r="I5" s="20" t="s">
+      <c r="I5" s="21" t="s">
         <v>215</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="J5" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="K5" s="21" t="s">
         <v>217</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="L5" s="21" t="s">
         <v>218</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="M5" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="N5" s="20" t="s">
+      <c r="N5" s="21" t="s">
         <v>220</v>
       </c>
-      <c r="O5" s="20" t="s">
+      <c r="O5" s="21" t="s">
         <v>221</v>
       </c>
-      <c r="P5" s="20" t="s">
+      <c r="P5" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="Q5" s="20" t="s">
+      <c r="Q5" s="21" t="s">
         <v>222</v>
       </c>
-      <c r="R5" s="20" t="s">
+      <c r="R5" s="21" t="s">
         <v>223</v>
       </c>
-      <c r="S5" s="20" t="s">
+      <c r="S5" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="T5" s="20" t="s">
+      <c r="T5" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="U5" s="20" t="s">
+      <c r="U5" s="21" t="s">
         <v>225</v>
       </c>
-      <c r="V5" s="20" t="s">
+      <c r="V5" s="21" t="s">
         <v>226</v>
       </c>
-      <c r="W5" s="20" t="s">
+      <c r="W5" s="21" t="s">
         <v>227</v>
       </c>
-      <c r="X5" s="20" t="s">
+      <c r="X5" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="Y5" s="20" t="s">
+      <c r="Y5" s="21" t="s">
         <v>229</v>
       </c>
-      <c r="Z5" s="20" t="s">
+      <c r="Z5" s="21" t="s">
         <v>230</v>
       </c>
-      <c r="AA5" s="20" t="s">
+      <c r="AA5" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="AB5" s="20" t="s">
+      <c r="AB5" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="AC5" s="20" t="s">
+      <c r="AC5" s="21" t="s">
         <v>232</v>
       </c>
-      <c r="AD5" s="20" t="s">
+      <c r="AD5" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="AE5" s="20" t="s">
+      <c r="AE5" s="21" t="s">
         <v>233</v>
       </c>
-      <c r="AF5" s="20" t="s">
+      <c r="AF5" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="AG5" s="20" t="s">
+      <c r="AG5" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="AH5" s="20" t="s">
+      <c r="AH5" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="AI5" s="20" t="s">
+      <c r="AI5" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="AJ5" s="20" t="s">
+      <c r="AJ5" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="AK5" s="20" t="s">
+      <c r="AK5" s="21" t="s">
         <v>235</v>
       </c>
-      <c r="AL5" s="20" t="s">
+      <c r="AL5" s="21" t="s">
         <v>236</v>
       </c>
-      <c r="AM5" s="20" t="s">
+      <c r="AM5" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="AN5" s="20" t="s">
+      <c r="AN5" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="AO5" s="20" t="s">
+      <c r="AO5" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="AP5" s="20" t="s">
+      <c r="AP5" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="AQ5" s="20" t="s">
+      <c r="AQ5" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="AR5" s="20" t="s">
+      <c r="AR5" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="AS5" s="20" t="s">
+      <c r="AS5" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="AT5" s="20" t="s">
+      <c r="AT5" s="21" t="s">
         <v>244</v>
       </c>
-      <c r="AU5" s="20" t="s">
+      <c r="AU5" s="21" t="s">
         <v>245</v>
       </c>
-      <c r="AV5" s="20" t="s">
+      <c r="AV5" s="21" t="s">
         <v>246</v>
       </c>
-      <c r="AW5" s="20" t="s">
+      <c r="AW5" s="21" t="s">
         <v>247</v>
       </c>
-      <c r="AX5" s="20" t="s">
+      <c r="AX5" s="21" t="s">
         <v>248</v>
       </c>
-      <c r="AY5" s="20" t="s">
+      <c r="AY5" s="21" t="s">
         <v>249</v>
       </c>
-      <c r="AZ5" s="20" t="s">
+      <c r="AZ5" s="21" t="s">
         <v>250</v>
       </c>
-      <c r="BA5" s="20" t="s">
+      <c r="BA5" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="BB5" s="20" t="s">
+      <c r="BB5" s="21" t="s">
         <v>252</v>
       </c>
-      <c r="BC5" s="20" t="s">
+      <c r="BC5" s="21" t="s">
         <v>253</v>
       </c>
-      <c r="BD5" s="20" t="s">
+      <c r="BD5" s="21" t="s">
         <v>254</v>
       </c>
-      <c r="BE5" s="20" t="s">
+      <c r="BE5" s="21" t="s">
         <v>255</v>
       </c>
-      <c r="BF5" s="20" t="s">
+      <c r="BF5" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="BG5" s="20" t="s">
+      <c r="BG5" s="21" t="s">
         <v>257</v>
       </c>
-      <c r="BH5" s="20" t="s">
+      <c r="BH5" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="BI5" s="20" t="s">
+      <c r="BI5" s="21" t="s">
         <v>259</v>
       </c>
-      <c r="BJ5" s="20" t="s">
+      <c r="BJ5" s="21" t="s">
         <v>260</v>
       </c>
-      <c r="BK5" s="20" t="s">
+      <c r="BK5" s="21" t="s">
         <v>261</v>
       </c>
-      <c r="BL5" s="20" t="s">
+      <c r="BL5" s="21" t="s">
         <v>262</v>
       </c>
-      <c r="BM5" s="20" t="s">
+      <c r="BM5" s="21" t="s">
         <v>263</v>
       </c>
-      <c r="BN5" s="20" t="s">
+      <c r="BN5" s="21" t="s">
         <v>264</v>
       </c>
-      <c r="BO5" s="20" t="s">
+      <c r="BO5" s="21" t="s">
         <v>265</v>
       </c>
-      <c r="BP5" s="20" t="s">
+      <c r="BP5" s="21" t="s">
         <v>266</v>
       </c>
-      <c r="BQ5" s="20" t="s">
+      <c r="BQ5" s="21" t="s">
         <v>267</v>
       </c>
-      <c r="BR5" s="20" t="s">
+      <c r="BR5" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="BS5" s="20" t="s">
+      <c r="BS5" s="21" t="s">
         <v>269</v>
       </c>
-      <c r="BT5" s="20" t="s">
+      <c r="BT5" s="21" t="s">
         <v>270</v>
       </c>
-      <c r="BU5" s="20" t="s">
+      <c r="BU5" s="21" t="s">
         <v>271</v>
       </c>
-      <c r="BV5" s="20" t="s">
+      <c r="BV5" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="BW5" s="20" t="s">
+      <c r="BW5" s="21" t="s">
         <v>273</v>
       </c>
-      <c r="BX5" s="20" t="s">
+      <c r="BX5" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="BY5" s="20" t="s">
+      <c r="BY5" s="21" t="s">
         <v>275</v>
       </c>
-      <c r="BZ5" s="20" t="s">
+      <c r="BZ5" s="21" t="s">
         <v>276</v>
       </c>
-      <c r="CA5" s="20" t="s">
+      <c r="CA5" s="21" t="s">
         <v>277</v>
       </c>
-      <c r="CB5" s="20" t="s">
+      <c r="CB5" s="21" t="s">
         <v>278</v>
       </c>
-      <c r="CC5" s="20" t="s">
+      <c r="CC5" s="21" t="s">
         <v>279</v>
       </c>
-      <c r="CD5" s="20" t="s">
+      <c r="CD5" s="21" t="s">
         <v>280</v>
       </c>
-      <c r="CE5" s="20" t="s">
+      <c r="CE5" s="21" t="s">
         <v>281</v>
       </c>
-      <c r="CF5" s="20" t="s">
+      <c r="CF5" s="21" t="s">
         <v>282</v>
       </c>
-      <c r="CG5" s="20" t="s">
+      <c r="CG5" s="21" t="s">
         <v>283</v>
       </c>
-      <c r="CH5" s="20" t="s">
+      <c r="CH5" s="21" t="s">
         <v>284</v>
       </c>
-      <c r="CI5" s="20" t="s">
+      <c r="CI5" s="21" t="s">
         <v>285</v>
       </c>
-      <c r="CJ5" s="20" t="s">
+      <c r="CJ5" s="21" t="s">
         <v>286</v>
       </c>
-      <c r="CK5" s="20" t="s">
+      <c r="CK5" s="21" t="s">
         <v>287</v>
       </c>
-      <c r="CL5" s="20" t="s">
+      <c r="CL5" s="21" t="s">
         <v>288</v>
       </c>
-      <c r="CM5" s="20" t="s">
+      <c r="CM5" s="21" t="s">
         <v>289</v>
       </c>
-      <c r="CN5" s="20" t="s">
+      <c r="CN5" s="21" t="s">
         <v>290</v>
       </c>
-      <c r="CO5" s="20" t="s">
+      <c r="CO5" s="21" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="22" t="s">
         <v>117</v>
       </c>
       <c r="B6" s="13" t="str">
         <f t="shared" ref="B6:CO6" si="1">TEXT(MOD(TIMEVALUE(B5)+3/1440,1),"HH:MM")</f>
-        <v>01:03</v>
+        <v>02:03</v>
       </c>
       <c r="C6" s="13" t="str">
         <f t="shared" si="1"/>
@@ -29834,12 +29834,12 @@
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="23" t="s">
         <v>116</v>
       </c>
       <c r="B7" s="15" t="str">
         <f t="shared" ref="B7:CO7" si="2">TEXT(MOD(TIMEVALUE(B5)+5/1440,1),"HH:MM")</f>
-        <v>01:05</v>
+        <v>02:05</v>
       </c>
       <c r="C7" s="15" t="str">
         <f t="shared" si="2"/>
@@ -30207,12 +30207,12 @@
       </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>115</v>
       </c>
       <c r="B8" s="13" t="str">
         <f t="shared" ref="B8:CO8" si="3">TEXT(MOD(TIMEVALUE(B5)+7/1440,1),"HH:MM")</f>
-        <v>01:07</v>
+        <v>02:07</v>
       </c>
       <c r="C8" s="13" t="str">
         <f t="shared" si="3"/>
@@ -30580,12 +30580,12 @@
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="23" t="s">
         <v>114</v>
       </c>
       <c r="B9" s="15" t="str">
         <f t="shared" ref="B9:CO9" si="4">TEXT(MOD(TIMEVALUE(B5)+9/1440,1),"HH:MM")</f>
-        <v>01:09</v>
+        <v>02:09</v>
       </c>
       <c r="C9" s="15" t="str">
         <f t="shared" si="4"/>
@@ -30953,12 +30953,12 @@
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>113</v>
       </c>
       <c r="B10" s="13" t="str">
         <f t="shared" ref="B10:CO10" si="5">TEXT(MOD(TIMEVALUE(B5)+11/1440,1),"HH:MM")</f>
-        <v>01:11</v>
+        <v>02:11</v>
       </c>
       <c r="C10" s="13" t="str">
         <f t="shared" si="5"/>
@@ -31326,12 +31326,12 @@
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="23" t="s">
         <v>112</v>
       </c>
       <c r="B11" s="15" t="str">
         <f t="shared" ref="B11:CO11" si="6">TEXT(MOD(TIMEVALUE(B5)+13/1440,1),"HH:MM")</f>
-        <v>01:13</v>
+        <v>02:13</v>
       </c>
       <c r="C11" s="15" t="str">
         <f t="shared" si="6"/>
@@ -31699,12 +31699,12 @@
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="22" t="s">
         <v>111</v>
       </c>
       <c r="B12" s="13" t="str">
         <f t="shared" ref="B12:CO12" si="7">TEXT(MOD(TIMEVALUE(B5)+15/1440,1),"HH:MM")</f>
-        <v>01:15</v>
+        <v>02:15</v>
       </c>
       <c r="C12" s="13" t="str">
         <f t="shared" si="7"/>
@@ -32072,12 +32072,12 @@
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="23" t="s">
         <v>110</v>
       </c>
       <c r="B13" s="15" t="str">
         <f t="shared" ref="B13:CO13" si="8">TEXT(MOD(TIMEVALUE(B5)+17/1440,1),"HH:MM")</f>
-        <v>01:17</v>
+        <v>02:17</v>
       </c>
       <c r="C13" s="15" t="str">
         <f t="shared" si="8"/>
@@ -32445,12 +32445,12 @@
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>109</v>
       </c>
       <c r="B14" s="13" t="str">
         <f t="shared" ref="B14:CO14" si="9">TEXT(MOD(TIMEVALUE(B5)+19/1440,1),"HH:MM")</f>
-        <v>01:19</v>
+        <v>02:19</v>
       </c>
       <c r="C14" s="13" t="str">
         <f t="shared" si="9"/>
@@ -32818,12 +32818,12 @@
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="23" t="s">
         <v>108</v>
       </c>
       <c r="B15" s="15" t="str">
         <f t="shared" ref="B15:CO15" si="10">TEXT(MOD(TIMEVALUE(B5)+21/1440,1),"HH:MM")</f>
-        <v>01:21</v>
+        <v>02:21</v>
       </c>
       <c r="C15" s="15" t="str">
         <f t="shared" si="10"/>
@@ -33191,12 +33191,12 @@
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="22" t="s">
         <v>107</v>
       </c>
       <c r="B16" s="13" t="str">
         <f t="shared" ref="B16:CO16" si="11">TEXT(MOD(TIMEVALUE(B5)+24/1440,1),"HH:MM")</f>
-        <v>01:24</v>
+        <v>02:24</v>
       </c>
       <c r="C16" s="13" t="str">
         <f t="shared" si="11"/>
@@ -33564,12 +33564,12 @@
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="23" t="s">
         <v>106</v>
       </c>
       <c r="B17" s="15" t="str">
         <f t="shared" ref="B17:CO17" si="12">TEXT(MOD(TIMEVALUE(B5)+26/1440,1),"HH:MM")</f>
-        <v>01:26</v>
+        <v>02:26</v>
       </c>
       <c r="C17" s="15" t="str">
         <f t="shared" si="12"/>
@@ -33937,12 +33937,12 @@
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="22" t="s">
         <v>105</v>
       </c>
       <c r="B18" s="13" t="str">
         <f t="shared" ref="B18:CO18" si="13">TEXT(MOD(TIMEVALUE(B5)+28/1440,1),"HH:MM")</f>
-        <v>01:28</v>
+        <v>02:28</v>
       </c>
       <c r="C18" s="13" t="str">
         <f t="shared" si="13"/>
@@ -34310,12 +34310,12 @@
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="23" t="s">
         <v>104</v>
       </c>
       <c r="B19" s="15" t="str">
         <f t="shared" ref="B19:CO19" si="14">TEXT(MOD(TIMEVALUE(B5)+29/1440,1),"HH:MM")</f>
-        <v>01:29</v>
+        <v>02:29</v>
       </c>
       <c r="C19" s="15" t="str">
         <f t="shared" si="14"/>
@@ -34683,12 +34683,12 @@
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>103</v>
       </c>
       <c r="B20" s="13" t="str">
         <f t="shared" ref="B20:CO20" si="15">TEXT(MOD(TIMEVALUE(B5)+33/1440,1),"HH:MM")</f>
-        <v>01:33</v>
+        <v>02:33</v>
       </c>
       <c r="C20" s="13" t="str">
         <f t="shared" si="15"/>
@@ -35056,12 +35056,12 @@
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="23" t="s">
         <v>102</v>
       </c>
       <c r="B21" s="15" t="str">
         <f t="shared" ref="B21:CO21" si="16">TEXT(MOD(TIMEVALUE(B5)+34/1440,1),"HH:MM")</f>
-        <v>01:34</v>
+        <v>02:34</v>
       </c>
       <c r="C21" s="15" t="str">
         <f t="shared" si="16"/>
@@ -35429,12 +35429,12 @@
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>101</v>
       </c>
       <c r="B22" s="13" t="str">
         <f t="shared" ref="B22:CO22" si="17">TEXT(MOD(TIMEVALUE(B5)+37/1440,1),"HH:MM")</f>
-        <v>01:37</v>
+        <v>02:37</v>
       </c>
       <c r="C22" s="13" t="str">
         <f t="shared" si="17"/>
@@ -35802,12 +35802,12 @@
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="23" t="s">
         <v>100</v>
       </c>
       <c r="B23" s="15" t="str">
         <f t="shared" ref="B23:CO23" si="18">TEXT(MOD(TIMEVALUE(B5)+39/1440,1),"HH:MM")</f>
-        <v>01:39</v>
+        <v>02:39</v>
       </c>
       <c r="C23" s="15" t="str">
         <f t="shared" si="18"/>
@@ -36175,12 +36175,12 @@
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="22" t="s">
         <v>99</v>
       </c>
       <c r="B24" s="13" t="str">
         <f t="shared" ref="B24:CO24" si="19">TEXT(MOD(TIMEVALUE(B5)+41/1440,1),"HH:MM")</f>
-        <v>01:41</v>
+        <v>02:41</v>
       </c>
       <c r="C24" s="13" t="str">
         <f t="shared" si="19"/>
@@ -36548,12 +36548,12 @@
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="23" t="s">
         <v>98</v>
       </c>
       <c r="B25" s="15" t="str">
         <f t="shared" ref="B25:CO25" si="20">TEXT(MOD(TIMEVALUE(B5)+43/1440,1),"HH:MM")</f>
-        <v>01:43</v>
+        <v>02:43</v>
       </c>
       <c r="C25" s="15" t="str">
         <f t="shared" si="20"/>
@@ -36921,12 +36921,12 @@
       </c>
     </row>
     <row r="26" ht="16.5" customHeight="1">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="22" t="s">
         <v>97</v>
       </c>
       <c r="B26" s="13" t="str">
         <f t="shared" ref="B26:CO26" si="21">TEXT(MOD(TIMEVALUE(B5)+45/1440,1),"HH:MM")</f>
-        <v>01:45</v>
+        <v>02:45</v>
       </c>
       <c r="C26" s="13" t="str">
         <f t="shared" si="21"/>
@@ -37294,12 +37294,12 @@
       </c>
     </row>
     <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="23" t="s">
         <v>95</v>
       </c>
       <c r="B27" s="15" t="str">
         <f t="shared" ref="B27:CO27" si="22">TEXT(MOD(TIMEVALUE(B5)+48/1440,1),"HH:MM")</f>
-        <v>01:48</v>
+        <v>02:48</v>
       </c>
       <c r="C27" s="15" t="str">
         <f t="shared" si="22"/>
@@ -38758,139 +38758,139 @@
       <c r="A1" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="23"/>
-      <c r="AB1" s="23"/>
-      <c r="AC1" s="23"/>
-      <c r="AD1" s="23"/>
-      <c r="AE1" s="23"/>
-      <c r="AF1" s="23"/>
-      <c r="AG1" s="23"/>
-      <c r="AH1" s="23"/>
-      <c r="AI1" s="23"/>
-      <c r="AJ1" s="23"/>
-      <c r="AK1" s="23"/>
-      <c r="AL1" s="23"/>
-      <c r="AM1" s="23"/>
-      <c r="AN1" s="23"/>
-      <c r="AO1" s="23"/>
-      <c r="AP1" s="23"/>
-      <c r="AQ1" s="23"/>
-      <c r="AR1" s="23"/>
-      <c r="AS1" s="23"/>
-      <c r="AT1" s="23"/>
-      <c r="AU1" s="23"/>
-      <c r="AV1" s="23"/>
-      <c r="AW1" s="23"/>
-      <c r="AX1" s="23"/>
-      <c r="AY1" s="23"/>
-      <c r="AZ1" s="23"/>
-      <c r="BA1" s="23"/>
-      <c r="BB1" s="23"/>
-      <c r="BC1" s="23"/>
-      <c r="BD1" s="23"/>
-      <c r="BE1" s="23"/>
-      <c r="BF1" s="23"/>
-      <c r="BG1" s="23"/>
-      <c r="BH1" s="23"/>
-      <c r="BI1" s="23"/>
-      <c r="BJ1" s="23"/>
-      <c r="BK1" s="23"/>
-      <c r="BL1" s="23"/>
-      <c r="BM1" s="24"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="24"/>
+      <c r="S1" s="24"/>
+      <c r="T1" s="24"/>
+      <c r="U1" s="24"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="24"/>
+      <c r="AA1" s="24"/>
+      <c r="AB1" s="24"/>
+      <c r="AC1" s="24"/>
+      <c r="AD1" s="24"/>
+      <c r="AE1" s="24"/>
+      <c r="AF1" s="24"/>
+      <c r="AG1" s="24"/>
+      <c r="AH1" s="24"/>
+      <c r="AI1" s="24"/>
+      <c r="AJ1" s="24"/>
+      <c r="AK1" s="24"/>
+      <c r="AL1" s="24"/>
+      <c r="AM1" s="24"/>
+      <c r="AN1" s="24"/>
+      <c r="AO1" s="24"/>
+      <c r="AP1" s="24"/>
+      <c r="AQ1" s="24"/>
+      <c r="AR1" s="24"/>
+      <c r="AS1" s="24"/>
+      <c r="AT1" s="24"/>
+      <c r="AU1" s="24"/>
+      <c r="AV1" s="24"/>
+      <c r="AW1" s="24"/>
+      <c r="AX1" s="24"/>
+      <c r="AY1" s="24"/>
+      <c r="AZ1" s="24"/>
+      <c r="BA1" s="24"/>
+      <c r="BB1" s="24"/>
+      <c r="BC1" s="24"/>
+      <c r="BD1" s="24"/>
+      <c r="BE1" s="24"/>
+      <c r="BF1" s="24"/>
+      <c r="BG1" s="24"/>
+      <c r="BH1" s="24"/>
+      <c r="BI1" s="24"/>
+      <c r="BJ1" s="24"/>
+      <c r="BK1" s="24"/>
+      <c r="BL1" s="24"/>
+      <c r="BM1" s="25"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
-      <c r="AA2" s="23"/>
-      <c r="AB2" s="23"/>
-      <c r="AC2" s="23"/>
-      <c r="AD2" s="23"/>
-      <c r="AE2" s="23"/>
-      <c r="AF2" s="23"/>
-      <c r="AG2" s="23"/>
-      <c r="AH2" s="23"/>
-      <c r="AI2" s="23"/>
-      <c r="AJ2" s="23"/>
-      <c r="AK2" s="23"/>
-      <c r="AL2" s="23"/>
-      <c r="AM2" s="23"/>
-      <c r="AN2" s="23"/>
-      <c r="AO2" s="23"/>
-      <c r="AP2" s="23"/>
-      <c r="AQ2" s="23"/>
-      <c r="AR2" s="23"/>
-      <c r="AS2" s="23"/>
-      <c r="AT2" s="23"/>
-      <c r="AU2" s="23"/>
-      <c r="AV2" s="23"/>
-      <c r="AW2" s="23"/>
-      <c r="AX2" s="23"/>
-      <c r="AY2" s="23"/>
-      <c r="AZ2" s="23"/>
-      <c r="BA2" s="23"/>
-      <c r="BB2" s="23"/>
-      <c r="BC2" s="23"/>
-      <c r="BD2" s="23"/>
-      <c r="BE2" s="23"/>
-      <c r="BF2" s="23"/>
-      <c r="BG2" s="23"/>
-      <c r="BH2" s="23"/>
-      <c r="BI2" s="23"/>
-      <c r="BJ2" s="23"/>
-      <c r="BK2" s="23"/>
-      <c r="BL2" s="23"/>
-      <c r="BM2" s="24"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="24"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="24"/>
+      <c r="T2" s="24"/>
+      <c r="U2" s="24"/>
+      <c r="V2" s="24"/>
+      <c r="W2" s="24"/>
+      <c r="X2" s="24"/>
+      <c r="Y2" s="24"/>
+      <c r="Z2" s="24"/>
+      <c r="AA2" s="24"/>
+      <c r="AB2" s="24"/>
+      <c r="AC2" s="24"/>
+      <c r="AD2" s="24"/>
+      <c r="AE2" s="24"/>
+      <c r="AF2" s="24"/>
+      <c r="AG2" s="24"/>
+      <c r="AH2" s="24"/>
+      <c r="AI2" s="24"/>
+      <c r="AJ2" s="24"/>
+      <c r="AK2" s="24"/>
+      <c r="AL2" s="24"/>
+      <c r="AM2" s="24"/>
+      <c r="AN2" s="24"/>
+      <c r="AO2" s="24"/>
+      <c r="AP2" s="24"/>
+      <c r="AQ2" s="24"/>
+      <c r="AR2" s="24"/>
+      <c r="AS2" s="24"/>
+      <c r="AT2" s="24"/>
+      <c r="AU2" s="24"/>
+      <c r="AV2" s="24"/>
+      <c r="AW2" s="24"/>
+      <c r="AX2" s="24"/>
+      <c r="AY2" s="24"/>
+      <c r="AZ2" s="24"/>
+      <c r="BA2" s="24"/>
+      <c r="BB2" s="24"/>
+      <c r="BC2" s="24"/>
+      <c r="BD2" s="24"/>
+      <c r="BE2" s="24"/>
+      <c r="BF2" s="24"/>
+      <c r="BG2" s="24"/>
+      <c r="BH2" s="24"/>
+      <c r="BI2" s="24"/>
+      <c r="BJ2" s="24"/>
+      <c r="BK2" s="24"/>
+      <c r="BL2" s="24"/>
+      <c r="BM2" s="25"/>
     </row>
     <row r="3" ht="4.5" customHeight="1"/>
     <row r="4" ht="19.5" customHeight="1">
@@ -39094,201 +39094,201 @@
       <c r="A5" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="21" t="s">
         <v>210</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="21" t="s">
         <v>294</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="20" t="s">
+      <c r="I5" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="J5" s="21" t="s">
         <v>296</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="K5" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="L5" s="21" t="s">
         <v>298</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="M5" s="21" t="s">
         <v>299</v>
       </c>
-      <c r="N5" s="20" t="s">
+      <c r="N5" s="21" t="s">
         <v>300</v>
       </c>
-      <c r="O5" s="20" t="s">
+      <c r="O5" s="21" t="s">
         <v>301</v>
       </c>
-      <c r="P5" s="20" t="s">
+      <c r="P5" s="21" t="s">
         <v>302</v>
       </c>
-      <c r="Q5" s="20" t="s">
+      <c r="Q5" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="R5" s="20" t="s">
+      <c r="R5" s="21" t="s">
         <v>304</v>
       </c>
-      <c r="S5" s="20" t="s">
+      <c r="S5" s="21" t="s">
         <v>305</v>
       </c>
-      <c r="T5" s="20" t="s">
+      <c r="T5" s="21" t="s">
         <v>306</v>
       </c>
-      <c r="U5" s="20" t="s">
+      <c r="U5" s="21" t="s">
         <v>307</v>
       </c>
-      <c r="V5" s="20" t="s">
+      <c r="V5" s="21" t="s">
         <v>308</v>
       </c>
-      <c r="W5" s="20" t="s">
+      <c r="W5" s="21" t="s">
         <v>309</v>
       </c>
-      <c r="X5" s="20" t="s">
+      <c r="X5" s="21" t="s">
         <v>310</v>
       </c>
-      <c r="Y5" s="20" t="s">
+      <c r="Y5" s="21" t="s">
         <v>311</v>
       </c>
-      <c r="Z5" s="20" t="s">
+      <c r="Z5" s="21" t="s">
         <v>235</v>
       </c>
-      <c r="AA5" s="20" t="s">
+      <c r="AA5" s="21" t="s">
         <v>236</v>
       </c>
-      <c r="AB5" s="20" t="s">
+      <c r="AB5" s="21" t="s">
         <v>237</v>
       </c>
-      <c r="AC5" s="20" t="s">
+      <c r="AC5" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="AD5" s="20" t="s">
+      <c r="AD5" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="AE5" s="20" t="s">
+      <c r="AE5" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="AF5" s="20" t="s">
+      <c r="AF5" s="21" t="s">
         <v>241</v>
       </c>
-      <c r="AG5" s="20" t="s">
+      <c r="AG5" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="AH5" s="20" t="s">
+      <c r="AH5" s="21" t="s">
         <v>312</v>
       </c>
-      <c r="AI5" s="20" t="s">
+      <c r="AI5" s="21" t="s">
         <v>313</v>
       </c>
-      <c r="AJ5" s="20" t="s">
+      <c r="AJ5" s="21" t="s">
         <v>246</v>
       </c>
-      <c r="AK5" s="20" t="s">
+      <c r="AK5" s="21" t="s">
         <v>314</v>
       </c>
-      <c r="AL5" s="20" t="s">
+      <c r="AL5" s="21" t="s">
         <v>315</v>
       </c>
-      <c r="AM5" s="20" t="s">
+      <c r="AM5" s="21" t="s">
         <v>250</v>
       </c>
-      <c r="AN5" s="20" t="s">
+      <c r="AN5" s="21" t="s">
         <v>316</v>
       </c>
-      <c r="AO5" s="20" t="s">
+      <c r="AO5" s="21" t="s">
         <v>317</v>
       </c>
-      <c r="AP5" s="20" t="s">
+      <c r="AP5" s="21" t="s">
         <v>254</v>
       </c>
-      <c r="AQ5" s="20" t="s">
+      <c r="AQ5" s="21" t="s">
         <v>318</v>
       </c>
-      <c r="AR5" s="20" t="s">
+      <c r="AR5" s="21" t="s">
         <v>319</v>
       </c>
-      <c r="AS5" s="20" t="s">
+      <c r="AS5" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="AT5" s="20" t="s">
+      <c r="AT5" s="21" t="s">
         <v>320</v>
       </c>
-      <c r="AU5" s="20" t="s">
+      <c r="AU5" s="21" t="s">
         <v>321</v>
       </c>
-      <c r="AV5" s="20" t="s">
+      <c r="AV5" s="21" t="s">
         <v>262</v>
       </c>
-      <c r="AW5" s="20" t="s">
+      <c r="AW5" s="21" t="s">
         <v>264</v>
       </c>
-      <c r="AX5" s="20" t="s">
+      <c r="AX5" s="21" t="s">
         <v>266</v>
       </c>
-      <c r="AY5" s="20" t="s">
+      <c r="AY5" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="AZ5" s="20" t="s">
+      <c r="AZ5" s="21" t="s">
         <v>270</v>
       </c>
-      <c r="BA5" s="20" t="s">
+      <c r="BA5" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="BB5" s="20" t="s">
+      <c r="BB5" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="BC5" s="20" t="s">
+      <c r="BC5" s="21" t="s">
         <v>276</v>
       </c>
-      <c r="BD5" s="20" t="s">
+      <c r="BD5" s="21" t="s">
         <v>278</v>
       </c>
-      <c r="BE5" s="20" t="s">
+      <c r="BE5" s="21" t="s">
         <v>280</v>
       </c>
-      <c r="BF5" s="20" t="s">
+      <c r="BF5" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="BG5" s="20" t="s">
+      <c r="BG5" s="21" t="s">
         <v>322</v>
       </c>
-      <c r="BH5" s="20" t="s">
+      <c r="BH5" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="BI5" s="20" t="s">
+      <c r="BI5" s="21" t="s">
         <v>323</v>
       </c>
-      <c r="BJ5" s="20" t="s">
+      <c r="BJ5" s="21" t="s">
         <v>324</v>
       </c>
-      <c r="BK5" s="20" t="s">
+      <c r="BK5" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="BL5" s="20" t="s">
+      <c r="BL5" s="21" t="s">
         <v>325</v>
       </c>
-      <c r="BM5" s="20" t="s">
+      <c r="BM5" s="21" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="22" t="s">
         <v>117</v>
       </c>
       <c r="B6" s="13" t="str">
@@ -39549,7 +39549,7 @@
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="23" t="s">
         <v>116</v>
       </c>
       <c r="B7" s="15" t="str">
@@ -39810,7 +39810,7 @@
       </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>115</v>
       </c>
       <c r="B8" s="13" t="str">
@@ -40071,7 +40071,7 @@
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="23" t="s">
         <v>114</v>
       </c>
       <c r="B9" s="15" t="str">
@@ -40332,7 +40332,7 @@
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>113</v>
       </c>
       <c r="B10" s="13" t="str">
@@ -40593,7 +40593,7 @@
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="23" t="s">
         <v>112</v>
       </c>
       <c r="B11" s="15" t="str">
@@ -40854,7 +40854,7 @@
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="22" t="s">
         <v>111</v>
       </c>
       <c r="B12" s="13" t="str">
@@ -41115,7 +41115,7 @@
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="23" t="s">
         <v>110</v>
       </c>
       <c r="B13" s="15" t="str">
@@ -41376,7 +41376,7 @@
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>109</v>
       </c>
       <c r="B14" s="13" t="str">
@@ -41637,7 +41637,7 @@
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="23" t="s">
         <v>108</v>
       </c>
       <c r="B15" s="15" t="str">
@@ -41898,7 +41898,7 @@
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="22" t="s">
         <v>107</v>
       </c>
       <c r="B16" s="13" t="str">
@@ -42159,7 +42159,7 @@
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="23" t="s">
         <v>106</v>
       </c>
       <c r="B17" s="15" t="str">
@@ -42420,7 +42420,7 @@
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="22" t="s">
         <v>105</v>
       </c>
       <c r="B18" s="13" t="str">
@@ -42681,7 +42681,7 @@
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="23" t="s">
         <v>104</v>
       </c>
       <c r="B19" s="15" t="str">
@@ -42942,7 +42942,7 @@
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>103</v>
       </c>
       <c r="B20" s="13" t="str">
@@ -43203,7 +43203,7 @@
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="23" t="s">
         <v>102</v>
       </c>
       <c r="B21" s="15" t="str">
@@ -43464,7 +43464,7 @@
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>101</v>
       </c>
       <c r="B22" s="13" t="str">
@@ -43725,7 +43725,7 @@
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="23" t="s">
         <v>100</v>
       </c>
       <c r="B23" s="15" t="str">
@@ -43986,7 +43986,7 @@
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="22" t="s">
         <v>99</v>
       </c>
       <c r="B24" s="13" t="str">
@@ -44247,7 +44247,7 @@
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="23" t="s">
         <v>98</v>
       </c>
       <c r="B25" s="15" t="str">
@@ -44508,7 +44508,7 @@
       </c>
     </row>
     <row r="26" ht="16.5" customHeight="1">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="22" t="s">
         <v>97</v>
       </c>
       <c r="B26" s="13" t="str">
@@ -44769,7 +44769,7 @@
       </c>
     </row>
     <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="23" t="s">
         <v>95</v>
       </c>
       <c r="B27" s="15" t="str">
@@ -46034,87 +46034,87 @@
       <c r="A1" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="23"/>
-      <c r="AB1" s="23"/>
-      <c r="AC1" s="23"/>
-      <c r="AD1" s="23"/>
-      <c r="AE1" s="23"/>
-      <c r="AF1" s="23"/>
-      <c r="AG1" s="23"/>
-      <c r="AH1" s="23"/>
-      <c r="AI1" s="23"/>
-      <c r="AJ1" s="23"/>
-      <c r="AK1" s="23"/>
-      <c r="AL1" s="23"/>
-      <c r="AM1" s="24"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="24"/>
+      <c r="S1" s="24"/>
+      <c r="T1" s="24"/>
+      <c r="U1" s="24"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="24"/>
+      <c r="AA1" s="24"/>
+      <c r="AB1" s="24"/>
+      <c r="AC1" s="24"/>
+      <c r="AD1" s="24"/>
+      <c r="AE1" s="24"/>
+      <c r="AF1" s="24"/>
+      <c r="AG1" s="24"/>
+      <c r="AH1" s="24"/>
+      <c r="AI1" s="24"/>
+      <c r="AJ1" s="24"/>
+      <c r="AK1" s="24"/>
+      <c r="AL1" s="24"/>
+      <c r="AM1" s="25"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
-      <c r="AA2" s="23"/>
-      <c r="AB2" s="23"/>
-      <c r="AC2" s="23"/>
-      <c r="AD2" s="23"/>
-      <c r="AE2" s="23"/>
-      <c r="AF2" s="23"/>
-      <c r="AG2" s="23"/>
-      <c r="AH2" s="23"/>
-      <c r="AI2" s="23"/>
-      <c r="AJ2" s="23"/>
-      <c r="AK2" s="23"/>
-      <c r="AL2" s="23"/>
-      <c r="AM2" s="24"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="24"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="24"/>
+      <c r="T2" s="24"/>
+      <c r="U2" s="24"/>
+      <c r="V2" s="24"/>
+      <c r="W2" s="24"/>
+      <c r="X2" s="24"/>
+      <c r="Y2" s="24"/>
+      <c r="Z2" s="24"/>
+      <c r="AA2" s="24"/>
+      <c r="AB2" s="24"/>
+      <c r="AC2" s="24"/>
+      <c r="AD2" s="24"/>
+      <c r="AE2" s="24"/>
+      <c r="AF2" s="24"/>
+      <c r="AG2" s="24"/>
+      <c r="AH2" s="24"/>
+      <c r="AI2" s="24"/>
+      <c r="AJ2" s="24"/>
+      <c r="AK2" s="24"/>
+      <c r="AL2" s="24"/>
+      <c r="AM2" s="25"/>
     </row>
     <row r="3" ht="4.5" customHeight="1"/>
     <row r="4" ht="19.5" customHeight="1">
@@ -46240,123 +46240,123 @@
       <c r="A5" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="21" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="21" t="s">
         <v>327</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="I5" s="20" t="s">
+      <c r="I5" s="21" t="s">
         <v>176</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="J5" s="21" t="s">
         <v>177</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="K5" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="L5" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="M5" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="N5" s="20" t="s">
+      <c r="N5" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="O5" s="20" t="s">
+      <c r="O5" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="P5" s="20" t="s">
+      <c r="P5" s="21" t="s">
         <v>183</v>
       </c>
-      <c r="Q5" s="20" t="s">
+      <c r="Q5" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="R5" s="20" t="s">
+      <c r="R5" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="S5" s="20" t="s">
+      <c r="S5" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="T5" s="20" t="s">
+      <c r="T5" s="21" t="s">
         <v>187</v>
       </c>
-      <c r="U5" s="20" t="s">
+      <c r="U5" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="V5" s="20" t="s">
+      <c r="V5" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="W5" s="20" t="s">
+      <c r="W5" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="X5" s="20" t="s">
+      <c r="X5" s="21" t="s">
         <v>191</v>
       </c>
-      <c r="Y5" s="20" t="s">
+      <c r="Y5" s="21" t="s">
         <v>192</v>
       </c>
-      <c r="Z5" s="20" t="s">
+      <c r="Z5" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="AA5" s="20" t="s">
+      <c r="AA5" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="AB5" s="20" t="s">
+      <c r="AB5" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="AC5" s="20" t="s">
+      <c r="AC5" s="21" t="s">
         <v>196</v>
       </c>
-      <c r="AD5" s="20" t="s">
+      <c r="AD5" s="21" t="s">
         <v>197</v>
       </c>
-      <c r="AE5" s="20" t="s">
+      <c r="AE5" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="AF5" s="20" t="s">
+      <c r="AF5" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="AG5" s="20" t="s">
+      <c r="AG5" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="AH5" s="20" t="s">
+      <c r="AH5" s="21" t="s">
         <v>201</v>
       </c>
-      <c r="AI5" s="20" t="s">
+      <c r="AI5" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="AJ5" s="20" t="s">
+      <c r="AJ5" s="21" t="s">
         <v>203</v>
       </c>
-      <c r="AK5" s="20" t="s">
+      <c r="AK5" s="21" t="s">
         <v>204</v>
       </c>
-      <c r="AL5" s="20" t="s">
+      <c r="AL5" s="21" t="s">
         <v>205</v>
       </c>
-      <c r="AM5" s="20" t="s">
+      <c r="AM5" s="21" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="22" t="s">
         <v>117</v>
       </c>
       <c r="B6" s="13" t="str">
@@ -46513,7 +46513,7 @@
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="23" t="s">
         <v>116</v>
       </c>
       <c r="B7" s="15" t="str">
@@ -46670,7 +46670,7 @@
       </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>115</v>
       </c>
       <c r="B8" s="13" t="str">
@@ -46827,7 +46827,7 @@
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="23" t="s">
         <v>114</v>
       </c>
       <c r="B9" s="15" t="str">
@@ -46984,7 +46984,7 @@
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>113</v>
       </c>
       <c r="B10" s="13" t="str">
@@ -47141,7 +47141,7 @@
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="23" t="s">
         <v>112</v>
       </c>
       <c r="B11" s="15" t="str">
@@ -47298,7 +47298,7 @@
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="22" t="s">
         <v>111</v>
       </c>
       <c r="B12" s="13" t="str">
@@ -47455,7 +47455,7 @@
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="23" t="s">
         <v>110</v>
       </c>
       <c r="B13" s="15" t="str">
@@ -47612,7 +47612,7 @@
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>109</v>
       </c>
       <c r="B14" s="13" t="str">
@@ -47769,7 +47769,7 @@
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="23" t="s">
         <v>108</v>
       </c>
       <c r="B15" s="15" t="str">
@@ -47926,7 +47926,7 @@
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="22" t="s">
         <v>107</v>
       </c>
       <c r="B16" s="13" t="str">
@@ -48083,7 +48083,7 @@
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="23" t="s">
         <v>106</v>
       </c>
       <c r="B17" s="15" t="str">
@@ -48240,7 +48240,7 @@
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="22" t="s">
         <v>105</v>
       </c>
       <c r="B18" s="13" t="str">
@@ -48397,7 +48397,7 @@
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="23" t="s">
         <v>104</v>
       </c>
       <c r="B19" s="15" t="str">
@@ -48554,7 +48554,7 @@
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>103</v>
       </c>
       <c r="B20" s="13" t="str">
@@ -48711,7 +48711,7 @@
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="23" t="s">
         <v>102</v>
       </c>
       <c r="B21" s="15" t="str">
@@ -48868,7 +48868,7 @@
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>101</v>
       </c>
       <c r="B22" s="13" t="str">
@@ -49025,7 +49025,7 @@
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="23" t="s">
         <v>100</v>
       </c>
       <c r="B23" s="15" t="str">
@@ -49182,7 +49182,7 @@
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="22" t="s">
         <v>99</v>
       </c>
       <c r="B24" s="13" t="str">
@@ -49339,7 +49339,7 @@
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="23" t="s">
         <v>98</v>
       </c>
       <c r="B25" s="15" t="str">
@@ -49496,7 +49496,7 @@
       </c>
     </row>
     <row r="26" ht="16.5" customHeight="1">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="22" t="s">
         <v>97</v>
       </c>
       <c r="B26" s="13" t="str">
@@ -49653,7 +49653,7 @@
       </c>
     </row>
     <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="23" t="s">
         <v>95</v>
       </c>
       <c r="B27" s="15" t="str">
@@ -50814,87 +50814,87 @@
       <c r="A1" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="23"/>
-      <c r="AB1" s="23"/>
-      <c r="AC1" s="23"/>
-      <c r="AD1" s="23"/>
-      <c r="AE1" s="23"/>
-      <c r="AF1" s="23"/>
-      <c r="AG1" s="23"/>
-      <c r="AH1" s="23"/>
-      <c r="AI1" s="23"/>
-      <c r="AJ1" s="23"/>
-      <c r="AK1" s="23"/>
-      <c r="AL1" s="23"/>
-      <c r="AM1" s="24"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
+      <c r="R1" s="24"/>
+      <c r="S1" s="24"/>
+      <c r="T1" s="24"/>
+      <c r="U1" s="24"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="24"/>
+      <c r="AA1" s="24"/>
+      <c r="AB1" s="24"/>
+      <c r="AC1" s="24"/>
+      <c r="AD1" s="24"/>
+      <c r="AE1" s="24"/>
+      <c r="AF1" s="24"/>
+      <c r="AG1" s="24"/>
+      <c r="AH1" s="24"/>
+      <c r="AI1" s="24"/>
+      <c r="AJ1" s="24"/>
+      <c r="AK1" s="24"/>
+      <c r="AL1" s="24"/>
+      <c r="AM1" s="25"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
-      <c r="AA2" s="23"/>
-      <c r="AB2" s="23"/>
-      <c r="AC2" s="23"/>
-      <c r="AD2" s="23"/>
-      <c r="AE2" s="23"/>
-      <c r="AF2" s="23"/>
-      <c r="AG2" s="23"/>
-      <c r="AH2" s="23"/>
-      <c r="AI2" s="23"/>
-      <c r="AJ2" s="23"/>
-      <c r="AK2" s="23"/>
-      <c r="AL2" s="23"/>
-      <c r="AM2" s="24"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="24"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="24"/>
+      <c r="T2" s="24"/>
+      <c r="U2" s="24"/>
+      <c r="V2" s="24"/>
+      <c r="W2" s="24"/>
+      <c r="X2" s="24"/>
+      <c r="Y2" s="24"/>
+      <c r="Z2" s="24"/>
+      <c r="AA2" s="24"/>
+      <c r="AB2" s="24"/>
+      <c r="AC2" s="24"/>
+      <c r="AD2" s="24"/>
+      <c r="AE2" s="24"/>
+      <c r="AF2" s="24"/>
+      <c r="AG2" s="24"/>
+      <c r="AH2" s="24"/>
+      <c r="AI2" s="24"/>
+      <c r="AJ2" s="24"/>
+      <c r="AK2" s="24"/>
+      <c r="AL2" s="24"/>
+      <c r="AM2" s="25"/>
     </row>
     <row r="3" ht="4.5" customHeight="1"/>
     <row r="4" ht="19.5" customHeight="1">
@@ -51020,128 +51020,128 @@
       <c r="A5" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="B5" s="25">
-        <v>0.08333333333333333</v>
-      </c>
-      <c r="C5" s="20" t="s">
+      <c r="B5" s="20">
+        <v>0.041666666666666664</v>
+      </c>
+      <c r="C5" s="21" t="s">
         <v>327</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="I5" s="20" t="s">
+      <c r="I5" s="21" t="s">
         <v>176</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="J5" s="21" t="s">
         <v>177</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="K5" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="L5" s="20" t="s">
+      <c r="L5" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="M5" s="20" t="s">
+      <c r="M5" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="N5" s="20" t="s">
+      <c r="N5" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="O5" s="20" t="s">
+      <c r="O5" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="P5" s="20" t="s">
+      <c r="P5" s="21" t="s">
         <v>183</v>
       </c>
-      <c r="Q5" s="20" t="s">
+      <c r="Q5" s="21" t="s">
         <v>184</v>
       </c>
-      <c r="R5" s="20" t="s">
+      <c r="R5" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="S5" s="20" t="s">
+      <c r="S5" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="T5" s="20" t="s">
+      <c r="T5" s="21" t="s">
         <v>187</v>
       </c>
-      <c r="U5" s="20" t="s">
+      <c r="U5" s="21" t="s">
         <v>188</v>
       </c>
-      <c r="V5" s="20" t="s">
+      <c r="V5" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="W5" s="20" t="s">
+      <c r="W5" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="X5" s="20" t="s">
+      <c r="X5" s="21" t="s">
         <v>191</v>
       </c>
-      <c r="Y5" s="20" t="s">
+      <c r="Y5" s="21" t="s">
         <v>192</v>
       </c>
-      <c r="Z5" s="20" t="s">
+      <c r="Z5" s="21" t="s">
         <v>193</v>
       </c>
-      <c r="AA5" s="20" t="s">
+      <c r="AA5" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="AB5" s="20" t="s">
+      <c r="AB5" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="AC5" s="20" t="s">
+      <c r="AC5" s="21" t="s">
         <v>196</v>
       </c>
-      <c r="AD5" s="20" t="s">
+      <c r="AD5" s="21" t="s">
         <v>197</v>
       </c>
-      <c r="AE5" s="20" t="s">
+      <c r="AE5" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="AF5" s="20" t="s">
+      <c r="AF5" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="AG5" s="20" t="s">
+      <c r="AG5" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="AH5" s="20" t="s">
+      <c r="AH5" s="21" t="s">
         <v>201</v>
       </c>
-      <c r="AI5" s="20" t="s">
+      <c r="AI5" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="AJ5" s="20" t="s">
+      <c r="AJ5" s="21" t="s">
         <v>203</v>
       </c>
-      <c r="AK5" s="20" t="s">
+      <c r="AK5" s="21" t="s">
         <v>204</v>
       </c>
-      <c r="AL5" s="20" t="s">
+      <c r="AL5" s="21" t="s">
         <v>205</v>
       </c>
-      <c r="AM5" s="20" t="s">
+      <c r="AM5" s="21" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="22" t="s">
         <v>117</v>
       </c>
       <c r="B6" s="13" t="str">
         <f t="shared" ref="B6:AM6" si="1">TEXT(MOD(TIMEVALUE(B5)+3/1440,1),"HH:MM")</f>
-        <v>02:03</v>
+        <v>01:03</v>
       </c>
       <c r="C6" s="13" t="str">
         <f t="shared" si="1"/>
@@ -51293,12 +51293,12 @@
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="23" t="s">
         <v>116</v>
       </c>
       <c r="B7" s="15" t="str">
         <f t="shared" ref="B7:AM7" si="2">TEXT(MOD(TIMEVALUE(B5)+5/1440,1),"HH:MM")</f>
-        <v>02:05</v>
+        <v>01:05</v>
       </c>
       <c r="C7" s="15" t="str">
         <f t="shared" si="2"/>
@@ -51450,12 +51450,12 @@
       </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>115</v>
       </c>
       <c r="B8" s="13" t="str">
         <f t="shared" ref="B8:AM8" si="3">TEXT(MOD(TIMEVALUE(B5)+7/1440,1),"HH:MM")</f>
-        <v>02:07</v>
+        <v>01:07</v>
       </c>
       <c r="C8" s="13" t="str">
         <f t="shared" si="3"/>
@@ -51607,12 +51607,12 @@
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="23" t="s">
         <v>114</v>
       </c>
       <c r="B9" s="15" t="str">
         <f t="shared" ref="B9:AM9" si="4">TEXT(MOD(TIMEVALUE(B5)+9/1440,1),"HH:MM")</f>
-        <v>02:09</v>
+        <v>01:09</v>
       </c>
       <c r="C9" s="15" t="str">
         <f t="shared" si="4"/>
@@ -51764,12 +51764,12 @@
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>113</v>
       </c>
       <c r="B10" s="13" t="str">
         <f t="shared" ref="B10:AM10" si="5">TEXT(MOD(TIMEVALUE(B5)+11/1440,1),"HH:MM")</f>
-        <v>02:11</v>
+        <v>01:11</v>
       </c>
       <c r="C10" s="13" t="str">
         <f t="shared" si="5"/>
@@ -51921,12 +51921,12 @@
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="23" t="s">
         <v>112</v>
       </c>
       <c r="B11" s="15" t="str">
         <f t="shared" ref="B11:AM11" si="6">TEXT(MOD(TIMEVALUE(B5)+13/1440,1),"HH:MM")</f>
-        <v>02:13</v>
+        <v>01:13</v>
       </c>
       <c r="C11" s="15" t="str">
         <f t="shared" si="6"/>
@@ -52078,12 +52078,12 @@
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="22" t="s">
         <v>111</v>
       </c>
       <c r="B12" s="13" t="str">
         <f t="shared" ref="B12:AM12" si="7">TEXT(MOD(TIMEVALUE(B5)+15/1440,1),"HH:MM")</f>
-        <v>02:15</v>
+        <v>01:15</v>
       </c>
       <c r="C12" s="13" t="str">
         <f t="shared" si="7"/>
@@ -52235,12 +52235,12 @@
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="23" t="s">
         <v>110</v>
       </c>
       <c r="B13" s="15" t="str">
         <f t="shared" ref="B13:AM13" si="8">TEXT(MOD(TIMEVALUE(B5)+17/1440,1),"HH:MM")</f>
-        <v>02:17</v>
+        <v>01:17</v>
       </c>
       <c r="C13" s="15" t="str">
         <f t="shared" si="8"/>
@@ -52392,12 +52392,12 @@
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>109</v>
       </c>
       <c r="B14" s="13" t="str">
         <f t="shared" ref="B14:AM14" si="9">TEXT(MOD(TIMEVALUE(B5)+19/1440,1),"HH:MM")</f>
-        <v>02:19</v>
+        <v>01:19</v>
       </c>
       <c r="C14" s="13" t="str">
         <f t="shared" si="9"/>
@@ -52549,12 +52549,12 @@
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="23" t="s">
         <v>108</v>
       </c>
       <c r="B15" s="15" t="str">
         <f t="shared" ref="B15:AM15" si="10">TEXT(MOD(TIMEVALUE(B5)+21/1440,1),"HH:MM")</f>
-        <v>02:21</v>
+        <v>01:21</v>
       </c>
       <c r="C15" s="15" t="str">
         <f t="shared" si="10"/>
@@ -52706,12 +52706,12 @@
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="22" t="s">
         <v>107</v>
       </c>
       <c r="B16" s="13" t="str">
         <f t="shared" ref="B16:AM16" si="11">TEXT(MOD(TIMEVALUE(B5)+24/1440,1),"HH:MM")</f>
-        <v>02:24</v>
+        <v>01:24</v>
       </c>
       <c r="C16" s="13" t="str">
         <f t="shared" si="11"/>
@@ -52863,12 +52863,12 @@
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="23" t="s">
         <v>106</v>
       </c>
       <c r="B17" s="15" t="str">
         <f t="shared" ref="B17:AM17" si="12">TEXT(MOD(TIMEVALUE(B5)+26/1440,1),"HH:MM")</f>
-        <v>02:26</v>
+        <v>01:26</v>
       </c>
       <c r="C17" s="15" t="str">
         <f t="shared" si="12"/>
@@ -53020,12 +53020,12 @@
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="22" t="s">
         <v>105</v>
       </c>
       <c r="B18" s="13" t="str">
         <f t="shared" ref="B18:AM18" si="13">TEXT(MOD(TIMEVALUE(B5)+28/1440,1),"HH:MM")</f>
-        <v>02:28</v>
+        <v>01:28</v>
       </c>
       <c r="C18" s="13" t="str">
         <f t="shared" si="13"/>
@@ -53177,12 +53177,12 @@
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="23" t="s">
         <v>104</v>
       </c>
       <c r="B19" s="15" t="str">
         <f t="shared" ref="B19:AM19" si="14">TEXT(MOD(TIMEVALUE(B5)+29/1440,1),"HH:MM")</f>
-        <v>02:29</v>
+        <v>01:29</v>
       </c>
       <c r="C19" s="15" t="str">
         <f t="shared" si="14"/>
@@ -53334,12 +53334,12 @@
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>103</v>
       </c>
       <c r="B20" s="13" t="str">
         <f t="shared" ref="B20:AM20" si="15">TEXT(MOD(TIMEVALUE(B5)+33/1440,1),"HH:MM")</f>
-        <v>02:33</v>
+        <v>01:33</v>
       </c>
       <c r="C20" s="13" t="str">
         <f t="shared" si="15"/>
@@ -53491,12 +53491,12 @@
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="23" t="s">
         <v>102</v>
       </c>
       <c r="B21" s="15" t="str">
         <f t="shared" ref="B21:AM21" si="16">TEXT(MOD(TIMEVALUE(B5)+34/1440,1),"HH:MM")</f>
-        <v>02:34</v>
+        <v>01:34</v>
       </c>
       <c r="C21" s="15" t="str">
         <f t="shared" si="16"/>
@@ -53648,12 +53648,12 @@
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>101</v>
       </c>
       <c r="B22" s="13" t="str">
         <f t="shared" ref="B22:AM22" si="17">TEXT(MOD(TIMEVALUE(B5)+37/1440,1),"HH:MM")</f>
-        <v>02:37</v>
+        <v>01:37</v>
       </c>
       <c r="C22" s="13" t="str">
         <f t="shared" si="17"/>
@@ -53805,12 +53805,12 @@
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="23" t="s">
         <v>100</v>
       </c>
       <c r="B23" s="15" t="str">
         <f t="shared" ref="B23:AM23" si="18">TEXT(MOD(TIMEVALUE(B5)+39/1440,1),"HH:MM")</f>
-        <v>02:39</v>
+        <v>01:39</v>
       </c>
       <c r="C23" s="15" t="str">
         <f t="shared" si="18"/>
@@ -53962,12 +53962,12 @@
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="22" t="s">
         <v>99</v>
       </c>
       <c r="B24" s="13" t="str">
         <f t="shared" ref="B24:AM24" si="19">TEXT(MOD(TIMEVALUE(B5)+41/1440,1),"HH:MM")</f>
-        <v>02:41</v>
+        <v>01:41</v>
       </c>
       <c r="C24" s="13" t="str">
         <f t="shared" si="19"/>
@@ -54119,12 +54119,12 @@
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="23" t="s">
         <v>98</v>
       </c>
       <c r="B25" s="15" t="str">
         <f t="shared" ref="B25:AM25" si="20">TEXT(MOD(TIMEVALUE(B5)+43/1440,1),"HH:MM")</f>
-        <v>02:43</v>
+        <v>01:43</v>
       </c>
       <c r="C25" s="15" t="str">
         <f t="shared" si="20"/>
@@ -54276,12 +54276,12 @@
       </c>
     </row>
     <row r="26" ht="16.5" customHeight="1">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="22" t="s">
         <v>97</v>
       </c>
       <c r="B26" s="13" t="str">
         <f t="shared" ref="B26:AM26" si="21">TEXT(MOD(TIMEVALUE(B5)+45/1440,1),"HH:MM")</f>
-        <v>02:45</v>
+        <v>01:45</v>
       </c>
       <c r="C26" s="13" t="str">
         <f t="shared" si="21"/>
@@ -54433,12 +54433,12 @@
       </c>
     </row>
     <row r="27" ht="16.5" customHeight="1">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="23" t="s">
         <v>95</v>
       </c>
       <c r="B27" s="15" t="str">
         <f t="shared" ref="B27:AM27" si="22">TEXT(MOD(TIMEVALUE(B5)+48/1440,1),"HH:MM")</f>
-        <v>02:48</v>
+        <v>01:48</v>
       </c>
       <c r="C27" s="15" t="str">
         <f t="shared" si="22"/>

</xml_diff>

<commit_message>
test #4 workflow horarios
</commit_message>
<xml_diff>
--- a/tren-urquiza-horarios.xlsx
+++ b/tren-urquiza-horarios.xlsx
@@ -29184,7 +29184,7 @@
         <v>118</v>
       </c>
       <c r="B5" s="20">
-        <v>0.08333333333333333</v>
+        <v>0.041666666666666664</v>
       </c>
       <c r="C5" s="21" t="s">
         <v>210</v>
@@ -29466,7 +29466,7 @@
       </c>
       <c r="B6" s="13" t="str">
         <f t="shared" ref="B6:CO6" si="1">TEXT(MOD(TIMEVALUE(B5)+3/1440,1),"HH:MM")</f>
-        <v>02:03</v>
+        <v>01:03</v>
       </c>
       <c r="C6" s="13" t="str">
         <f t="shared" si="1"/>
@@ -29839,7 +29839,7 @@
       </c>
       <c r="B7" s="15" t="str">
         <f t="shared" ref="B7:CO7" si="2">TEXT(MOD(TIMEVALUE(B5)+5/1440,1),"HH:MM")</f>
-        <v>02:05</v>
+        <v>01:05</v>
       </c>
       <c r="C7" s="15" t="str">
         <f t="shared" si="2"/>
@@ -30212,7 +30212,7 @@
       </c>
       <c r="B8" s="13" t="str">
         <f t="shared" ref="B8:CO8" si="3">TEXT(MOD(TIMEVALUE(B5)+7/1440,1),"HH:MM")</f>
-        <v>02:07</v>
+        <v>01:07</v>
       </c>
       <c r="C8" s="13" t="str">
         <f t="shared" si="3"/>
@@ -30585,7 +30585,7 @@
       </c>
       <c r="B9" s="15" t="str">
         <f t="shared" ref="B9:CO9" si="4">TEXT(MOD(TIMEVALUE(B5)+9/1440,1),"HH:MM")</f>
-        <v>02:09</v>
+        <v>01:09</v>
       </c>
       <c r="C9" s="15" t="str">
         <f t="shared" si="4"/>
@@ -30958,7 +30958,7 @@
       </c>
       <c r="B10" s="13" t="str">
         <f t="shared" ref="B10:CO10" si="5">TEXT(MOD(TIMEVALUE(B5)+11/1440,1),"HH:MM")</f>
-        <v>02:11</v>
+        <v>01:11</v>
       </c>
       <c r="C10" s="13" t="str">
         <f t="shared" si="5"/>
@@ -31331,7 +31331,7 @@
       </c>
       <c r="B11" s="15" t="str">
         <f t="shared" ref="B11:CO11" si="6">TEXT(MOD(TIMEVALUE(B5)+13/1440,1),"HH:MM")</f>
-        <v>02:13</v>
+        <v>01:13</v>
       </c>
       <c r="C11" s="15" t="str">
         <f t="shared" si="6"/>
@@ -31704,7 +31704,7 @@
       </c>
       <c r="B12" s="13" t="str">
         <f t="shared" ref="B12:CO12" si="7">TEXT(MOD(TIMEVALUE(B5)+15/1440,1),"HH:MM")</f>
-        <v>02:15</v>
+        <v>01:15</v>
       </c>
       <c r="C12" s="13" t="str">
         <f t="shared" si="7"/>
@@ -32077,7 +32077,7 @@
       </c>
       <c r="B13" s="15" t="str">
         <f t="shared" ref="B13:CO13" si="8">TEXT(MOD(TIMEVALUE(B5)+17/1440,1),"HH:MM")</f>
-        <v>02:17</v>
+        <v>01:17</v>
       </c>
       <c r="C13" s="15" t="str">
         <f t="shared" si="8"/>
@@ -32450,7 +32450,7 @@
       </c>
       <c r="B14" s="13" t="str">
         <f t="shared" ref="B14:CO14" si="9">TEXT(MOD(TIMEVALUE(B5)+19/1440,1),"HH:MM")</f>
-        <v>02:19</v>
+        <v>01:19</v>
       </c>
       <c r="C14" s="13" t="str">
         <f t="shared" si="9"/>
@@ -32823,7 +32823,7 @@
       </c>
       <c r="B15" s="15" t="str">
         <f t="shared" ref="B15:CO15" si="10">TEXT(MOD(TIMEVALUE(B5)+21/1440,1),"HH:MM")</f>
-        <v>02:21</v>
+        <v>01:21</v>
       </c>
       <c r="C15" s="15" t="str">
         <f t="shared" si="10"/>
@@ -33196,7 +33196,7 @@
       </c>
       <c r="B16" s="13" t="str">
         <f t="shared" ref="B16:CO16" si="11">TEXT(MOD(TIMEVALUE(B5)+24/1440,1),"HH:MM")</f>
-        <v>02:24</v>
+        <v>01:24</v>
       </c>
       <c r="C16" s="13" t="str">
         <f t="shared" si="11"/>
@@ -33569,7 +33569,7 @@
       </c>
       <c r="B17" s="15" t="str">
         <f t="shared" ref="B17:CO17" si="12">TEXT(MOD(TIMEVALUE(B5)+26/1440,1),"HH:MM")</f>
-        <v>02:26</v>
+        <v>01:26</v>
       </c>
       <c r="C17" s="15" t="str">
         <f t="shared" si="12"/>
@@ -33942,7 +33942,7 @@
       </c>
       <c r="B18" s="13" t="str">
         <f t="shared" ref="B18:CO18" si="13">TEXT(MOD(TIMEVALUE(B5)+28/1440,1),"HH:MM")</f>
-        <v>02:28</v>
+        <v>01:28</v>
       </c>
       <c r="C18" s="13" t="str">
         <f t="shared" si="13"/>
@@ -34315,7 +34315,7 @@
       </c>
       <c r="B19" s="15" t="str">
         <f t="shared" ref="B19:CO19" si="14">TEXT(MOD(TIMEVALUE(B5)+29/1440,1),"HH:MM")</f>
-        <v>02:29</v>
+        <v>01:29</v>
       </c>
       <c r="C19" s="15" t="str">
         <f t="shared" si="14"/>
@@ -34688,7 +34688,7 @@
       </c>
       <c r="B20" s="13" t="str">
         <f t="shared" ref="B20:CO20" si="15">TEXT(MOD(TIMEVALUE(B5)+33/1440,1),"HH:MM")</f>
-        <v>02:33</v>
+        <v>01:33</v>
       </c>
       <c r="C20" s="13" t="str">
         <f t="shared" si="15"/>
@@ -35061,7 +35061,7 @@
       </c>
       <c r="B21" s="15" t="str">
         <f t="shared" ref="B21:CO21" si="16">TEXT(MOD(TIMEVALUE(B5)+34/1440,1),"HH:MM")</f>
-        <v>02:34</v>
+        <v>01:34</v>
       </c>
       <c r="C21" s="15" t="str">
         <f t="shared" si="16"/>
@@ -35434,7 +35434,7 @@
       </c>
       <c r="B22" s="13" t="str">
         <f t="shared" ref="B22:CO22" si="17">TEXT(MOD(TIMEVALUE(B5)+37/1440,1),"HH:MM")</f>
-        <v>02:37</v>
+        <v>01:37</v>
       </c>
       <c r="C22" s="13" t="str">
         <f t="shared" si="17"/>
@@ -35807,7 +35807,7 @@
       </c>
       <c r="B23" s="15" t="str">
         <f t="shared" ref="B23:CO23" si="18">TEXT(MOD(TIMEVALUE(B5)+39/1440,1),"HH:MM")</f>
-        <v>02:39</v>
+        <v>01:39</v>
       </c>
       <c r="C23" s="15" t="str">
         <f t="shared" si="18"/>
@@ -36180,7 +36180,7 @@
       </c>
       <c r="B24" s="13" t="str">
         <f t="shared" ref="B24:CO24" si="19">TEXT(MOD(TIMEVALUE(B5)+41/1440,1),"HH:MM")</f>
-        <v>02:41</v>
+        <v>01:41</v>
       </c>
       <c r="C24" s="13" t="str">
         <f t="shared" si="19"/>
@@ -36553,7 +36553,7 @@
       </c>
       <c r="B25" s="15" t="str">
         <f t="shared" ref="B25:CO25" si="20">TEXT(MOD(TIMEVALUE(B5)+43/1440,1),"HH:MM")</f>
-        <v>02:43</v>
+        <v>01:43</v>
       </c>
       <c r="C25" s="15" t="str">
         <f t="shared" si="20"/>
@@ -36926,7 +36926,7 @@
       </c>
       <c r="B26" s="13" t="str">
         <f t="shared" ref="B26:CO26" si="21">TEXT(MOD(TIMEVALUE(B5)+45/1440,1),"HH:MM")</f>
-        <v>02:45</v>
+        <v>01:45</v>
       </c>
       <c r="C26" s="13" t="str">
         <f t="shared" si="21"/>
@@ -37299,7 +37299,7 @@
       </c>
       <c r="B27" s="15" t="str">
         <f t="shared" ref="B27:CO27" si="22">TEXT(MOD(TIMEVALUE(B5)+48/1440,1),"HH:MM")</f>
-        <v>02:48</v>
+        <v>01:48</v>
       </c>
       <c r="C27" s="15" t="str">
         <f t="shared" si="22"/>

</xml_diff>